<commit_message>
test cases + automation
</commit_message>
<xml_diff>
--- a/Test_Cases_QARO-59.xlsx
+++ b/Test_Cases_QARO-59.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="139">
   <si>
     <t>ID</t>
   </si>
@@ -37,40 +37,35 @@
     <t>Positive</t>
   </si>
   <si>
-    <t>Verify Login Form UI Elements Display</t>
-  </si>
-  <si>
-    <t>N/A</t>
+    <t>Verify presence of all required UI elements on Login Form</t>
+  </si>
+  <si>
+    <t>User is on the Login Page.</t>
   </si>
   <si>
     <t>1. Navigate to the Login Page.</t>
   </si>
   <si>
-    <t xml:space="preserve">The Login Form is displayed with:
-- Email input field.
-- Password input field.
-- Password Show/Hide toggle icon next to the Password field.
-- "Login" button.
-- "Forgot Password?" link.
-- A global notification area (initially empty).</t>
+    <t xml:space="preserve">The Login Form is displayed and includes:
+- Email input field
+- Password input field
+- 'Show/Hide' toggle icon next to the Password field
+- 'Login' button
+- 'Forgot Password?' link
+- A visible global notification area for security errors.</t>
   </si>
   <si>
     <t>TC002</t>
   </si>
   <si>
-    <t>Verify Password Field Toggle Icon Functionality</t>
-  </si>
-  <si>
-    <t>User is on the Login Page.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter a password (e.g., 'testpassword') into the Password field.
-2. Click the 'Show' icon (e.g., eye icon).
-3. Click the 'Hide' icon.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. After step 2, the entered password text is visible (e.g., 'testpassword'). The icon changes to 'Hide'.
-2. After step 3, the entered password text is masked (e.g., with asterisks or dots). The icon changes to 'Show'.</t>
+    <t>Verify email field accepts valid RFC 5322 format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter a valid email address conforming to RFC 5322 (e.g., 'test.user_alias%tag+2023@sub.domain-name.co.uk') in the Email field.
+2. Click outside the Email field to trigger 'On Blur' validation.</t>
+  </si>
+  <si>
+    <t>No inline error message appears below the Email field.</t>
   </si>
   <si>
     <t>TC003</t>
@@ -79,408 +74,412 @@
     <t>Negative</t>
   </si>
   <si>
-    <t>Verify Email Field 'Required' Inline Error on Blur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Focus on the Email input field.
-2. Leave the Email input field empty.
-3. Click into the Password input field (triggering 'On Blur' for Email).</t>
-  </si>
-  <si>
-    <t>An inline error message "This field is required." (ERR-VAL-01) appears in red below the Email field.</t>
+    <t>Verify email field rejects invalid format (missing '@' symbol)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'invalidemail.com' (missing '@') in the Email field.
+2. Click outside the Email field to trigger 'On Blur' validation.</t>
+  </si>
+  <si>
+    <t>An inline error message 'Please enter a valid email address (e.g., name@domain.com).' appears below the Email field (ERR-VAL-02).</t>
   </si>
   <si>
     <t>TC004</t>
   </si>
   <si>
-    <t>Verify Email Field 'Invalid Format' Inline Error (Missing @)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter "testexample.com" into the Email field.
-2. Click into the Password field (triggering 'On Blur').</t>
-  </si>
-  <si>
-    <t>An inline error message "Please enter a valid email address (e.g., name@domain.com)." (ERR-VAL-02) appears in red below the Email field.</t>
+    <t>Verify email field rejects invalid format (no domain part)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'user@' in the Email field.
+2. Click outside the Email field to trigger 'On Blur' validation.</t>
   </si>
   <si>
     <t>TC005</t>
   </si>
   <si>
-    <t>Verify Email Field 'Invalid Format' Inline Error (Missing Domain)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter "test@" into the Email field.
-2. Click into the Password field (triggering 'On Blur').</t>
+    <t>Verify email field rejects invalid characters in local part</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'user!name@domain.com' (invalid character '!') in the Email field.
+2. Click outside the Email field to trigger 'On Blur' validation.</t>
   </si>
   <si>
     <t>TC006</t>
   </si>
   <si>
-    <t>Verify Email Field 'Invalid Format' Inline Error (Invalid Characters)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter "user name@domain.com" into the Email field.
-2. Click into the Password field (triggering 'On Blur').</t>
+    <t>Edge Case</t>
+  </si>
+  <si>
+    <t>Verify email field accepts maximum allowed length (254 characters)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Generate a valid email address with exactly 254 characters (e.g., 'abcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklm@example.com').
+2. Enter this 254-character email into the Email field.
+3. Click outside the Email field to trigger 'On Blur' validation.</t>
+  </si>
+  <si>
+    <t>No inline error message appears below the Email field. The email is accepted.</t>
   </si>
   <si>
     <t>TC007</t>
   </si>
   <si>
-    <t>Verify Email Field Accepts Valid RFC 5322 Characters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter "name.surname+tag%01@sub.domain.co.uk" into the Email field.
-2. Click into the Password field (triggering 'On Blur').</t>
-  </si>
-  <si>
-    <t>No inline error message appears under the Email field.</t>
+    <t>Verify email field rejects input exceeding maximum allowed length (254 characters)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Generate a valid email address with 255 characters (e.g., 'abcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmnopqrstuvwxyzabcdefghijklmn@example.com').
+2. Enter this 255-character email into the Email field.
+3. Click outside the Email field to trigger 'On Blur' validation.</t>
+  </si>
+  <si>
+    <t>An inline error message 'Please enter a valid email address (e.g., name@domain.com).' appears below the Email field (ERR-VAL-02), indicating the length constraint is part of the format validation.</t>
   </si>
   <si>
     <t>TC008</t>
   </si>
   <si>
-    <t>Verify Email Field Trims Leading/Trailing Whitespaces</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter "  valid.email@example.com  " (with leading and trailing spaces) into the Email field.
-2. Click into the Password field (triggering 'On Blur').
-3. Observe the behavior of the input field (e.g., programmatically check its value or attempt to log in).</t>
-  </si>
-  <si>
-    <t>No inline error message appears. The Email field's value is internally treated as "valid.email@example.com" (leading/trailing spaces trimmed) for validation and submission.</t>
+    <t>Verify leading and trailing whitespaces are trimmed automatically from email input</t>
+  </si>
+  <si>
+    <t>User is on the Login Page. A valid user account exists (e.g., 'valid.user@example.com' with password 'SecurePass123!').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter '  valid.user@example.com  ' (with leading/trailing spaces) in the Email field.
+2. Enter 'SecurePass123!' in the Password field.
+3. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>User is successfully logged into their dashboard, indicating that leading and trailing whitespaces were trimmed from the email before validation and authentication.</t>
   </si>
   <si>
     <t>TC009</t>
   </si>
   <si>
-    <t>Edge Case</t>
-  </si>
-  <si>
-    <t>Verify Email Field Accepts Maximum Length (254 characters)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Construct a valid email address that is exactly 254 characters long (e.g., 'a.long.email.address.with.many.characters.to.reach.the.maximum.limit.of.two.hundred.fifty.four.characters.in.the.local.part.and.domain.part.of.an.email.address.example.com@testdomainforextremelongemails.co.uk').
-2. Enter this email into the Email field.
-3. Click into the Password field (triggering 'On Blur').</t>
-  </si>
-  <si>
-    <t>No inline error message appears under the Email field. The input is accepted.</t>
+    <t>Verify password field accepts full UTF-8 character set including space and special symbols</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter a password containing uppercase, lowercase, digits, spaces, special characters, and UTF-8 symbols (e.g., 'P@ssw0rd W!th Sp@ce &amp; UTF-8 chars £€😂') in the Password field.
+2. Click outside the Password field to trigger 'On Blur' validation.</t>
+  </si>
+  <si>
+    <t>No inline error message appears below the Password field. The Password field accepts all characters without issue.</t>
   </si>
   <si>
     <t>TC010</t>
   </si>
   <si>
-    <t>Verify Email Field Prevents Typing Beyond Maximum Length (254 characters)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Construct a string of 255 characters (e.g., 'a' repeated 255 times, or a valid email part that is 255 chars).
-2. Attempt to enter this 255-character string into the Email field.</t>
-  </si>
-  <si>
-    <t>The Email field only accepts the first 254 characters, preventing any further input. No inline error message appears as it's a prevention, not a validation error after input.</t>
+    <t>Verify password field accepts minimum allowed length (8 characters)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'MinPass!' (exactly 8 characters) in the Password field.
+2. Click outside the Password field to trigger 'On Blur' validation.</t>
+  </si>
+  <si>
+    <t>No inline error message appears below the Password field.</t>
   </si>
   <si>
     <t>TC011</t>
   </si>
   <si>
-    <t>Verify Password Field 'Required' Inline Error on Blur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter a valid email (e.g., 'test@example.com') into the Email input field.
-2. Focus on the Password input field.
-3. Leave the Password input field empty.
-4. Click anywhere outside the Password field (triggering 'On Blur').</t>
-  </si>
-  <si>
-    <t>An inline error message "This field is required." (ERR-VAL-01) appears in red below the Password field.</t>
+    <t>Verify password field accepts maximum allowed length (128 characters)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter a password with exactly 128 characters in the Password field.
+2. Click outside the Password field to trigger 'On Blur' validation.</t>
   </si>
   <si>
     <t>TC012</t>
   </si>
   <si>
-    <t>Verify Password Field 'Length Out of Bounds' Inline Error (Below Min)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter a valid email (e.g., 'test@example.com') into the Email field.
-2. Enter "P@ss123" (7 characters) into the Password field.
-3. Click anywhere outside the Password field (triggering 'On Blur').</t>
-  </si>
-  <si>
-    <t>An inline error message "Password must be between 8 and 128 characters." (ERR-VAL-03) appears in red below the Password field.</t>
+    <t>Verify password field rejects input less than minimum allowed length (7 characters)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'ShortP7' (7 characters) in the Password field.
+2. Click outside the Password field to trigger 'On Blur' validation.</t>
+  </si>
+  <si>
+    <t>An inline error message 'Password must be between 8 and 128 characters.' appears below the Password field (ERR-VAL-03).</t>
   </si>
   <si>
     <t>TC013</t>
   </si>
   <si>
-    <t>Verify Password Field 'Length Out of Bounds' Inline Error (Above Max)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter a valid email (e.g., 'test@example.com') into the Email field.
-2. Enter a password that is 129 characters long (e.g., 128 chars + 1).
-3. Click anywhere outside the Password field (triggering 'On Blur').</t>
+    <t>Verify password field rejects input exceeding maximum allowed length (129 characters)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter a password with 129 characters in the Password field.
+2. Click outside the Password field to trigger 'On Blur' validation.</t>
   </si>
   <si>
     <t>TC014</t>
   </si>
   <si>
-    <t>Verify Password Field Accepts Minimum Length (8 characters)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter a valid email (e.g., 'test@example.com') into the Email field.
-2. Enter "P@ssword" (8 characters) into the Password field.
-3. Click anywhere outside the Password field.</t>
-  </si>
-  <si>
-    <t>No inline error message appears under the Password field.</t>
+    <t>Verify inline error for empty email and password fields on Login button click</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Leave Email field empty.
+2. Leave Password field empty.
+3. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>An inline error message 'This field is required.' appears below both the Email and Password fields. No network request should be sent to the backend server (ERR-VAL-01).</t>
   </si>
   <si>
     <t>TC015</t>
   </si>
   <si>
-    <t>Verify Password Field Accepts Maximum Length (128 characters)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter a valid email (e.g., 'test@example.com') into the Email field.
-2. Enter a password that is exactly 128 characters long, including various UTF-8, special characters, and spaces.
-3. Click anywhere outside the Password field.</t>
+    <t>Verify inline error for empty email field only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Leave Email field empty.
+2. Enter a valid password (e.g., 'SecurePass123!') in the Password field.
+3. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>An inline error message 'This field is required.' appears below the Email field. No network request should be sent to the backend server (ERR-VAL-01).</t>
   </si>
   <si>
     <t>TC016</t>
   </si>
   <si>
-    <t>Verify Password Field Accepts Full UTF-8 Character Set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter a valid email (e.g., 'test@example.com') into the Email field.
-2. Enter a password containing a mix of uppercase, lowercase, digits, special characters, symbols, spaces, and various UTF-8 characters (e.g., 'Pä$$w0rd!@#$ %^&amp;*()_+-=[]{}|;:'",.&lt;&gt;/?`~한글漢字日本語').
-3. Click anywhere outside the Password field.</t>
-  </si>
-  <si>
-    <t>No inline error message appears under the Password field. The input is accepted.</t>
+    <t>Verify inline error for empty password field only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter a valid email (e.g., 'test@example.com') in the Email field.
+2. Leave Password field empty.
+3. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>An inline error message 'This field is required.' appears below the Password field. No network request should be sent to the backend server (ERR-VAL-01).</t>
   </si>
   <si>
     <t>TC017</t>
   </si>
   <si>
-    <t>Verify Inline Errors for Both Empty Email and Password on Login Click (AC1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Leave both Email and Password fields empty.
-2. Click the "Login" button.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. An inline error message "This field is required." (ERR-VAL-01) appears in red below the Email field.
-2. An inline error message "This field is required." (ERR-VAL-01) appears in red below the Password field.
-3. No request is sent to the backend server.</t>
+    <t>Verify inline error for malformed email on blur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'john.doe#domain.com' in the Email field.
+2. Click into the Password field (triggering 'On Blur' for Email field).</t>
   </si>
   <si>
     <t>TC018</t>
   </si>
   <si>
-    <t>Verify Inline Error for Malformed Email on Blur (AC2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter "john.doe#domain.com" in the Email field.
-2. Click into the Password field (triggering Blur).</t>
-  </si>
-  <si>
-    <t>An inline error "Please enter a valid email address (e.g., name@domain.com)." (ERR-VAL-02) appears in red under the Email field.</t>
+    <t>Verify inline error for password less than 8 characters on blur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'Pass123' (7 characters) in the Password field.
+2. Click into the Email field (triggering 'On Blur' for Password field).</t>
   </si>
   <si>
     <t>TC019</t>
   </si>
   <si>
-    <t>Successful Login with Valid Credentials</t>
-  </si>
-  <si>
-    <t>A registered user exists with email "user@test.com" and password "P@ssword123".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Navigate to the Login Page.
-2. Enter "user@test.com" in the Email field.
-3. Enter "P@ssword123" in the Password field.
-4. Click the "Login" button.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. The user is redirected to their dashboard or home page.
-2. No error messages are displayed.</t>
+    <t>Verify inline error for password more than 128 characters on blur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter a 129-character password in the Password field.
+2. Click into the Email field (triggering 'On Blur' for Password field).</t>
   </si>
   <si>
     <t>TC020</t>
   </si>
   <si>
-    <t>Generic Failure Message for Incorrect Password (AC3)</t>
-  </si>
-  <si>
-    <t>A registered user exists with email "existing_user@test.com" and password "CorrectP@ssword123".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Navigate to the Login Page.
-2. Enter "existing_user@test.com" in the Email field.
-3. Enter "IncorrectP@ssword" in the Password field.
-4. Click the "Login" button.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. A global alert message "Invalid email or password. Please try again." (ERR-AUTH-01) is displayed (Global Toast - Alert Red).
-2. The system must NOT disclose that the email "existing_user@test.com" exists (e.g., no different error message or response time).
-3. The login page remains displayed.
-4. Verify the server response time is identical to an unregistered user attempt (requires backend logging/monitoring).</t>
+    <t>Verify successful login with valid credentials</t>
+  </si>
+  <si>
+    <t>An account exists with email 'existing_user@test.com' and password 'SecurePass123!'. User is on the Login Page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'existing_user@test.com' in the Email field.
+2. Enter 'SecurePass123!' in the Password field.
+3. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>User is successfully authenticated and redirected to their dashboard.</t>
   </si>
   <si>
     <t>TC021</t>
   </si>
   <si>
-    <t>Generic Failure Message for Unregistered Email</t>
-  </si>
-  <si>
-    <t>An unregistered email "nonexistent@test.com" does not exist in the system.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Navigate to the Login Page.
-2. Enter "nonexistent@test.com" in the Email field.
-3. Enter "AnyP@ssword123" in the Password field.
-4. Click the "Login" button.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. A global alert message "Invalid email or password. Please try again." (ERR-AUTH-01) is displayed (Global Toast - Alert Red).
-2. The system must NOT disclose that the email "nonexistent@test.com" does not exist (e.g., no different error message or response time).
-3. The login page remains displayed.
-4. Verify the server response time is identical to a registered user with an incorrect password attempt (requires backend logging/monitoring).</t>
+    <t>Verify generic error message for incorrect password for an existing user (User Enumeration protection)</t>
+  </si>
+  <si>
+    <t>An account exists with email 'existing_user@test.com'. User is on the Login Page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'existing_user@test.com' in the Email field.
+2. Enter 'IncorrectPass123!' in the Password field.
+3. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>A global alert message (Toast - Alert Red) 'Invalid email or password. Please try again.' is displayed. The server response time for this request must be identical to attempts with non-existent emails to prevent user enumeration (ERR-AUTH-01).</t>
   </si>
   <si>
     <t>TC022</t>
   </si>
   <si>
-    <t>Account Lockout After 5 Failed Attempts (AC4 - 5th Attempt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. A registered account exists with email "user@test.com".
-2. The account is not currently locked.
-3. An IP address is associated with these attempts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Perform 4 consecutive failed login attempts for "user@test.com" (e.g., with wrong passwords), ensuring each attempt receives the "Invalid email or password" message.
-2. On the 5th attempt, enter "user@test.com" and an incorrect password.
-3. Click "Login".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. A global banner message: "Too many failed login attempts. For security reasons, your access has been locked for 15 minutes. You can reset your password to unlock it immediately." (ERR-AUTH-LOCK) is displayed (Global Banner - Dark Red).
-2. The user is unable to log in.
-3. Backend logs show 5 failed login attempts for "user@test.com" with masked email and IP address.</t>
+    <t>Verify generic error message for unregistered email (User Enumeration protection)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'nonexistent@example.com' in the Email field.
+2. Enter 'AnyValidPass123!' in the Password field.
+3. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>A global alert message (Toast - Alert Red) 'Invalid email or password. Please try again.' is displayed. The server response time for this request must be identical to attempts with existing emails and incorrect passwords to prevent user enumeration (ERR-AUTH-01).</t>
   </si>
   <si>
     <t>TC023</t>
   </si>
   <si>
-    <t>Blocked Subsequent Login Attempts After Lockout (AC4 - Subsequent Attempts)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. An account "user@test.com" is currently locked due to 5 failed attempts within the last 15 minutes.
-2. The 15-minute lockout period has not expired.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Attempt to log in with "user@test.com" and a correct password.
-2. Attempt to log in with "user@test.com" and an incorrect password.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. For both attempts, the global banner message: "Too many failed login attempts. For security reasons, your access has been locked for 15 minutes. You can reset your password to unlock it immediately." (ERR-AUTH-LOCK) is displayed.
-2. The request should be blocked at the API Gateway level (if applicable).
-3. No successful login occurs.</t>
+    <t>Verify account lockout after 5 consecutive failed login attempts for the same email (Rate Limiting)</t>
+  </si>
+  <si>
+    <t>An account exists with email 'user@test.com'. User is on the Login Page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Attempt to log in with 'user@test.com' and an incorrect password 4 times consecutively within 15 minutes.
+2. On the 5th attempt, enter 'user@test.com' and an incorrect password.
+3. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>On the 5th attempt, a global banner (Dark Red) 'Too many failed login attempts. For security reasons, your access has been locked for 15 minutes. You can reset your password to unlock it immediately.' is displayed (ERR-AUTH-LOCK).</t>
   </si>
   <si>
     <t>TC024</t>
   </si>
   <si>
-    <t>Account Unlock After 15 Minutes Timeout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. An account "user@test.com" was locked due to 5 failed attempts.
-2. More than 15 minutes have passed since the lockout occurred.</t>
-  </si>
-  <si>
-    <t>1. Attempt to log in with "user@test.com" and the correct password.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. The user successfully logs in and is redirected to their dashboard.
-2. No lockout message is displayed.</t>
+    <t>Verify login attempts are blocked during account lockout period</t>
+  </si>
+  <si>
+    <t>Account 'user@test.com' is currently locked due to rate limiting (e.g., from TC023). User is on the Login Page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Attempt to log in with 'user@test.com' and any password (correct or incorrect) within the 15-minute lockout period.
+2. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>A global banner (Dark Red) 'Too many failed login attempts. For security reasons, your access has been locked for 15 minutes. You can reset your password to unlock it immediately.' is displayed. The request should be blocked automatically at the API Gateway level, and no authentication attempt should reach the backend.</t>
   </si>
   <si>
     <t>TC025</t>
   </si>
   <si>
-    <t>SQL Injection Attempt in Email Field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter "admin' OR '1'='1" in the Email field.
-2. Enter any valid password (e.g., "password123") in the Password field.
-3. Click the "Login" button.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. A global message "Invalid request. Special characters detected." (ERR-SEC-01) is displayed.
-2. The request is blocked at the API Gateway level.
-3. No successful login occurs.</t>
+    <t>Verify system blocks SQL Injection patterns in Email field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'admin' OR '1'='1'--' in the Email field.
+2. Enter any valid password (e.g., 'SecurePass123!') in the Password field.
+3. Click the 'Login' button.</t>
+  </si>
+  <si>
+    <t>A global message 'Invalid request. Special characters detected.' is displayed. The request is blocked at the API Gateway level, preventing it from reaching the backend application (ERR-SEC-01).</t>
   </si>
   <si>
     <t>TC026</t>
   </si>
   <si>
-    <t>SQL Injection Attempt in Password Field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter a valid email (e.g., "test@example.com") in the Email field.
-2. Enter "' OR '1'='1" in the Password field.
-3. Click the "Login" button.</t>
+    <t>Verify system blocks XSS patterns in Email field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter '&lt;script&gt;alert("XSS")&lt;/script&gt;' in the Email field.
+2. Enter any valid password (e.g., 'SecurePass123!') in the Password field.
+3. Click the 'Login' button.</t>
   </si>
   <si>
     <t>TC027</t>
   </si>
   <si>
-    <t>XSS Attempt in Email Field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter `"&gt;&lt;script&gt;alert('XSS')&lt;/script&gt;` in the Email field.
-2. Enter a valid password (e.g., "password123") in the Password field.
-3. Click the "Login" button.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. A global message "Invalid request. Special characters detected." (ERR-SEC-01) is displayed.
-2. The request is blocked at the API Gateway level.
-3. No script execution occurs on the page.</t>
+    <t>Verify system blocks SQL Injection patterns in Password field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter a valid email (e.g., 'test@example.com') in the Email field.
+2. Enter 'password' OR '1'='1'--' in the Password field.
+3. Click the 'Login' button.</t>
   </si>
   <si>
     <t>TC028</t>
   </si>
   <si>
-    <t>XSS Attempt in Password Field</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Enter a valid email (e.g., "test@example.com") in the Email field.
-2. Enter `"&gt;&lt;script&gt;alert('XSS')&lt;/script&gt;` in the Password field.
-3. Click the "Login" button.</t>
+    <t>Verify system blocks XSS patterns in Password field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter a valid email (e.g., 'test@example.com') in the Email field.
+2. Enter '&lt;script&gt;alert("XSS")&lt;/script&gt;' in the Password field.
+3. Click the 'Login' button.</t>
   </si>
   <si>
     <t>TC029</t>
   </si>
   <si>
-    <t>Verify Telemetry Logging for Failed Login Attempts</t>
-  </si>
-  <si>
-    <t>A monitoring system is in place to view security audit logs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Navigate to the Login Page.
-2. Attempt to log in with an unregistered email "telemetrytest@example.com" and any password.
-3. Click "Login".
-4. Attempt to log in with a valid email "existing@example.com" and an incorrect password.
-5. Click "Login".
-6. Access the security audit logs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. For step 3, a global alert message "Invalid email or password. Please try again." is displayed.
-2. For step 5, a global alert message "Invalid email or password. Please try again." is displayed.
-3. In the security audit logs, two entries are found for failed login attempts.
-4. The IP address of the client making the request is logged for both attempts.
-5. The email addresses are masked (e.g., "t********t@example.com", "e********g@example.com").</t>
+    <t>Verify failed login attempts log masked email and IP in security audit logs</t>
+  </si>
+  <si>
+    <t>User is on the Login Page. Access to backend security audit logs is available.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Attempt to log in with an incorrect email or password (e.g., 'user@test.com' with 'wrongpass').
+2. Access the security audit logs in the backend monitoring system.
+3. Search for the failed login attempt based on the time and user.</t>
+  </si>
+  <si>
+    <t>A log entry for the failed login attempt is found, containing the IP address from which the attempt was made and the masked email address (e.g., 'u***r@test.com').</t>
+  </si>
+  <si>
+    <t>TC030</t>
+  </si>
+  <si>
+    <t>Verify password field content is initially hidden</t>
+  </si>
+  <si>
+    <t>1. Enter some characters (e.g., 'Password123') into the Password field.</t>
+  </si>
+  <si>
+    <t>The entered characters in the Password field are displayed as masked characters (e.g., asterisks or dots). A 'Show' toggle icon is visible.</t>
+  </si>
+  <si>
+    <t>TC031</t>
+  </si>
+  <si>
+    <t>Verify password field content becomes visible after clicking 'Show' toggle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'MySecretPass' in the Password field.
+2. Click the 'Show' toggle icon.</t>
+  </si>
+  <si>
+    <t>The text 'MySecretPass' is visible in the Password field. The toggle icon changes to indicate 'Hide' state.</t>
+  </si>
+  <si>
+    <t>TC032</t>
+  </si>
+  <si>
+    <t>Verify password field content becomes hidden after clicking 'Hide' toggle</t>
+  </si>
+  <si>
+    <t>User is on the Login Page. Password field is currently showing its content (e.g., after clicking 'Show').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Enter 'MySecretPass' in the Password field.
+2. Click the 'Show' toggle icon to reveal the content.
+3. Click the 'Hide' toggle icon.</t>
+  </si>
+  <si>
+    <t>The text 'MySecretPass' is hidden again (displayed as masked characters) in the Password field. The toggle icon changes back to indicate 'Show' state.</t>
+  </si>
+  <si>
+    <t>TC033</t>
+  </si>
+  <si>
+    <t>Verify 'Forgot Password?' link navigates to the correct page</t>
+  </si>
+  <si>
+    <t>1. Click the 'Forgot Password?' link.</t>
+  </si>
+  <si>
+    <t>The user is redirected to the 'Forgot Password' or password recovery page.</t>
   </si>
 </sst>
 </file>
@@ -874,7 +873,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -935,93 +934,93 @@
         <v>13</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="F5" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="F6" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1029,13 +1028,13 @@
         <v>32</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>33</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>34</v>
@@ -1055,27 +1054,27 @@
         <v>37</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>41</v>
+        <v>7</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>43</v>
@@ -1089,13 +1088,13 @@
         <v>45</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>46</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>47</v>
@@ -1109,99 +1108,99 @@
         <v>49</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>51</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="F14" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1209,13 +1208,13 @@
         <v>67</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>68</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>69</v>
@@ -1229,259 +1228,339 @@
         <v>71</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>73</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="F19" s="2" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="F20" s="2" t="s">
-        <v>83</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="23" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>96</v>
+        <v>9</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="28" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>119</v>
+        <v>107</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="F31" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="E30" s="2" t="s">
+    </row>
+    <row r="32" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="B32" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>127</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>